<commit_message>
chore: update model information and experimental predictions Excel files
</commit_message>
<xml_diff>
--- a/data/251114_model_vs_exp_pred.xlsx
+++ b/data/251114_model_vs_exp_pred.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -635,16 +635,16 @@
         <v>0.04633316489471607</v>
       </c>
       <c r="X2" t="n">
-        <v>0.04458054983482768</v>
+        <v>0.04458054983483162</v>
       </c>
       <c r="Y2" t="n">
         <v>-19.42112726586114</v>
       </c>
       <c r="Z2" t="n">
-        <v>-7.418641251971446</v>
+        <v>-7.418641251971524</v>
       </c>
       <c r="AA2" t="n">
-        <v>-2.129440016701112</v>
+        <v>-2.129440016701139</v>
       </c>
     </row>
     <row r="3">
@@ -718,16 +718,16 @@
         <v>0.04603843657912355</v>
       </c>
       <c r="X3" t="n">
-        <v>0.04317666445641467</v>
+        <v>0.04317666445641177</v>
       </c>
       <c r="Y3" t="n">
         <v>-19.14334128889219</v>
       </c>
       <c r="Z3" t="n">
-        <v>-7.351923154353286</v>
+        <v>-7.351923154353336</v>
       </c>
       <c r="AA3" t="n">
-        <v>-2.062381855356419</v>
+        <v>-2.062381855356439</v>
       </c>
     </row>
     <row r="4">
@@ -801,16 +801,16 @@
         <v>0.04610932025804834</v>
       </c>
       <c r="X4" t="n">
-        <v>0.04702037162974227</v>
+        <v>0.04702037162974387</v>
       </c>
       <c r="Y4" t="n">
         <v>-19.9038933743707</v>
       </c>
       <c r="Z4" t="n">
-        <v>-7.534591080345502</v>
+        <v>-7.534591080345474</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.24598084410148</v>
+        <v>-2.245980844101477</v>
       </c>
     </row>
     <row r="5">
@@ -888,7 +888,7 @@
         <v>0.03381414280423613</v>
       </c>
       <c r="X5" t="n">
-        <v>0.03430388907734183</v>
+        <v>0.03430388907734158</v>
       </c>
       <c r="Y5" t="n">
         <v>-17.38769042522724</v>
@@ -897,7 +897,7 @@
         <v>-6.930254332249933</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.638563777261961</v>
+        <v>-1.638563777261967</v>
       </c>
     </row>
     <row r="6">
@@ -971,16 +971,16 @@
         <v>0.03598329211613979</v>
       </c>
       <c r="X6" t="n">
-        <v>0.03474150091059358</v>
+        <v>0.03474150091059082</v>
       </c>
       <c r="Y6" t="n">
         <v>-17.47428042217543</v>
       </c>
       <c r="Z6" t="n">
-        <v>-6.951051349911411</v>
+        <v>-6.951051349911453</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.659466797815926</v>
+        <v>-1.659466797815944</v>
       </c>
     </row>
     <row r="7">
@@ -1054,16 +1054,16 @@
         <v>0.03598329211613979</v>
       </c>
       <c r="X7" t="n">
-        <v>0.03375693956402544</v>
+        <v>0.03375693956402783</v>
       </c>
       <c r="Y7" t="n">
         <v>-17.27946584561073</v>
       </c>
       <c r="Z7" t="n">
-        <v>-6.904261162449515</v>
+        <v>-6.90426116244948</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.612438119658331</v>
+        <v>-1.612438119658323</v>
       </c>
     </row>
     <row r="8">
@@ -1141,16 +1141,16 @@
         <v>0.02649065137240596</v>
       </c>
       <c r="X8" t="n">
-        <v>0.02441995144829998</v>
+        <v>0.02441995144829957</v>
       </c>
       <c r="Y8" t="n">
         <v>-15.43196147983211</v>
       </c>
       <c r="Z8" t="n">
-        <v>-6.460531144214263</v>
+        <v>-6.46053114421426</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.166446398991891</v>
+        <v>-1.166446398991897</v>
       </c>
     </row>
     <row r="9">
@@ -1224,16 +1224,16 @@
         <v>0.02629053704124418</v>
       </c>
       <c r="X9" t="n">
-        <v>0.02519588850012225</v>
+        <v>0.02519588850011989</v>
       </c>
       <c r="Y9" t="n">
         <v>-15.58549568947646</v>
       </c>
       <c r="Z9" t="n">
-        <v>-6.497406693147769</v>
+        <v>-6.497406693147809</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.203509903473277</v>
+        <v>-1.203509903473294</v>
       </c>
     </row>
     <row r="10">
@@ -1307,16 +1307,16 @@
         <v>0.02629053704124418</v>
       </c>
       <c r="X10" t="n">
-        <v>0.02661934966533718</v>
+        <v>0.0266193496653347</v>
       </c>
       <c r="Y10" t="n">
         <v>-15.86715511590536</v>
       </c>
       <c r="Z10" t="n">
-        <v>-6.565055108350689</v>
+        <v>-6.565055108350727</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.271503124253569</v>
+        <v>-1.271503124253587</v>
       </c>
     </row>
     <row r="11">
@@ -1394,16 +1394,16 @@
         <v>0.02082821603882547</v>
       </c>
       <c r="X11" t="n">
-        <v>0.02497042027184703</v>
+        <v>0.0249704202718446</v>
       </c>
       <c r="Y11" t="n">
         <v>-15.54088242330096</v>
       </c>
       <c r="Z11" t="n">
-        <v>-6.486691565335203</v>
+        <v>-6.486691565335234</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.192740160400012</v>
+        <v>-1.19274016040003</v>
       </c>
     </row>
     <row r="12">
@@ -1477,16 +1477,16 @@
         <v>0.0211696284081858</v>
       </c>
       <c r="X12" t="n">
-        <v>0.02220251933363635</v>
+        <v>0.0222025193336358</v>
       </c>
       <c r="Y12" t="n">
         <v>-14.99319948700468</v>
       </c>
       <c r="Z12" t="n">
-        <v>-6.355150139067756</v>
+        <v>-6.355150139067765</v>
       </c>
       <c r="AA12" t="n">
-        <v>-1.060528264361831</v>
+        <v>-1.060528264361836</v>
       </c>
     </row>
     <row r="13">
@@ -1560,16 +1560,439 @@
         <v>0.02017461580733303</v>
       </c>
       <c r="X13" t="n">
-        <v>0.02540530798341899</v>
+        <v>0.02540530798341969</v>
       </c>
       <c r="Y13" t="n">
         <v>-15.62693339989001</v>
       </c>
       <c r="Z13" t="n">
-        <v>-6.507359122131478</v>
+        <v>-6.507359122131469</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.213513060223627</v>
+        <v>-1.213513060223628</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF72-169 </t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1.900115681967213</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.690033283442623</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.3800102057377049</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2.562286104918033</v>
+      </c>
+      <c r="H14" t="n">
+        <v>6.714089742622951</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-1.185257140983607</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.0214988924567923</v>
+      </c>
+      <c r="K14" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2.277</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1.471904422781038</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.6033350766860873</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.12930603331976</v>
+      </c>
+      <c r="P14" t="n">
+        <v>11.3831070754539</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>4.665946833231703</v>
+      </c>
+      <c r="R14" t="n">
+        <v>2.43961354089622</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.4895297812411608</v>
+      </c>
+      <c r="T14" t="n">
+        <v>19.23876998218518</v>
+      </c>
+      <c r="U14" t="n">
+        <v>7.885990817675816</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1.690115875626869</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.0214988924567923</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.04365894563077947</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>-19.23876998218518</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>-7.374843032974132</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>-2.085418557142392</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF72-170 </t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1.900109978688524</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.6900407167213114</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.3800109350819671</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2.558167729508197</v>
+      </c>
+      <c r="H15" t="n">
+        <v>6.717556459016394</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-1.202454375409836</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.0214988924567923</v>
+      </c>
+      <c r="K15" t="n">
+        <v>39.35</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2.459</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.469181875741293</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.6022655927396198</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.1284153128305632</v>
+      </c>
+      <c r="P15" t="n">
+        <v>11.44086202305013</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>4.689982677800081</v>
+      </c>
+      <c r="R15" t="n">
+        <v>2.439425219458736</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.5286577655125226</v>
+      </c>
+      <c r="T15" t="n">
+        <v>17.78188331180518</v>
+      </c>
+      <c r="U15" t="n">
+        <v>7.289374222240213</v>
+      </c>
+      <c r="V15" t="n">
+        <v>1.554243314531691</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.0214988924567923</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0.03629607614085233</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>-17.78188331180518</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>-7.024930815829279</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>-1.733722829124487</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF72-171 </t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1.900124232786885</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.6900382363934426</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.3800155744262295</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2.562848121311475</v>
+      </c>
+      <c r="H16" t="n">
+        <v>6.710943296721311</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-1.189024496184956</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.0214988924567923</v>
+      </c>
+      <c r="K16" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.261</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1.480827951670002</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.605767936802129</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.1327723005442626</v>
+      </c>
+      <c r="P16" t="n">
+        <v>11.15313921352394</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>4.562457186619152</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2.444546602263808</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.4860899584480739</v>
+      </c>
+      <c r="T16" t="n">
+        <v>19.49237526155201</v>
+      </c>
+      <c r="U16" t="n">
+        <v>7.973820275506637</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1.747703035744069</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.0214988924567923</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0.04494062567624838</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>-19.49237526155201</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>-7.43575345750271</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>-2.146639443550002</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF72-178 </t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1.900126844262295</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.6900401929508198</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.3800132386885246</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.583189439344262</v>
+      </c>
+      <c r="H17" t="n">
+        <v>6.70666815409836</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-1.193879719672131</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.01869688457429442</v>
+      </c>
+      <c r="K17" t="n">
+        <v>41</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2.459</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1.453575231115186</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.6055309903959988</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.1155463809478317</v>
+      </c>
+      <c r="P17" t="n">
+        <v>12.58001522151926</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>5.240588112139933</v>
+      </c>
+      <c r="R17" t="n">
+        <v>2.400496843546508</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0.4597563916818998</v>
+      </c>
+      <c r="T17" t="n">
+        <v>17.59299210765102</v>
+      </c>
+      <c r="U17" t="n">
+        <v>7.328896163703775</v>
+      </c>
+      <c r="V17" t="n">
+        <v>1.398487346625512</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.01869688457429442</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0.035341450559976</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>-17.59299210765102</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>-6.979563292473808</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>-1.688124066426047</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SF72-182 </t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1.900136665573771</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.6900469359016392</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.380010504262295</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.591012770491803</v>
+      </c>
+      <c r="H18" t="n">
+        <v>6.711777754098361</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-1.162749909836066</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.01836711332099381</v>
+      </c>
+      <c r="K18" t="n">
+        <v>39.95</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2.455</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1.470649655219025</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.6069709790110251</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.126334925114212</v>
+      </c>
+      <c r="P18" t="n">
+        <v>11.64087962128839</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>4.804459087321249</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2.422932407106588</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0.4509126320303979</v>
+      </c>
+      <c r="T18" t="n">
+        <v>17.82864968503328</v>
+      </c>
+      <c r="U18" t="n">
+        <v>7.358294285363025</v>
+      </c>
+      <c r="V18" t="n">
+        <v>1.531555197291872</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.01836711332099381</v>
+      </c>
+      <c r="X18" t="n">
+        <v>0.03653242582377261</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>-17.82864968503328</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>-7.036163072721163</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>-1.745012337096256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>